<commit_message>
Check If a String Contains All Binary Codes of Size K.
</commit_message>
<xml_diff>
--- a/Pseudo.xlsx
+++ b/Pseudo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LC_Solutions\LC_Solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1441DB03-8B64-4A8B-BC16-F00667C1C7DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{888EB6BA-C122-431B-A97F-19DB11FFA559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="456">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="459">
   <si>
     <t>Id</t>
   </si>
@@ -1396,6 +1396,15 @@
   </si>
   <si>
     <t>Track prev index starting from -1 and find the max gap</t>
+  </si>
+  <si>
+    <t>Check If a String Contains All Binary Codes of Size K</t>
+  </si>
+  <si>
+    <t>Bitwise/Math/HashSet</t>
+  </si>
+  <si>
+    <t>HashSet to keep track, all = 2^k, iterate and check.</t>
   </si>
 </sst>
 </file>
@@ -1722,7 +1731,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G178"/>
+  <dimension ref="A1:G179"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -4227,6 +4236,20 @@
         <v>455</v>
       </c>
     </row>
+    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A179">
+        <v>1461</v>
+      </c>
+      <c r="B179" t="s">
+        <v>456</v>
+      </c>
+      <c r="C179" t="s">
+        <v>457</v>
+      </c>
+      <c r="D179" t="s">
+        <v>458</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G54">
     <sortCondition ref="A2:A54"/>

</xml_diff>

<commit_message>
Sum Of Root To Leaf Binary Numbers.
</commit_message>
<xml_diff>
--- a/Pseudo.xlsx
+++ b/Pseudo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LC_Solutions\LC_Solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{888EB6BA-C122-431B-A97F-19DB11FFA559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B289517E-390A-4014-86AD-060142EB7BE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="459">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="461">
   <si>
     <t>Id</t>
   </si>
@@ -1405,6 +1405,12 @@
   </si>
   <si>
     <t>HashSet to keep track, all = 2^k, iterate and check.</t>
+  </si>
+  <si>
+    <t>Sum of Root to Leaf Binary Numbers</t>
+  </si>
+  <si>
+    <t>Traverse all edges, collect the number and find the sum. (node == null return, left shift OR combo, if it's a leaf add to the sum, else recur)</t>
   </si>
 </sst>
 </file>
@@ -1731,7 +1737,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G179"/>
+  <dimension ref="A1:G180"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -4250,6 +4256,20 @@
         <v>458</v>
       </c>
     </row>
+    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A180">
+        <v>1022</v>
+      </c>
+      <c r="B180" t="s">
+        <v>459</v>
+      </c>
+      <c r="C180" t="s">
+        <v>449</v>
+      </c>
+      <c r="D180" t="s">
+        <v>460</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G54">
     <sortCondition ref="A2:A54"/>

</xml_diff>

<commit_message>
Sort Integers By The Number Of 1 Bits.
</commit_message>
<xml_diff>
--- a/Pseudo.xlsx
+++ b/Pseudo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LC_Solutions\LC_Solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B289517E-390A-4014-86AD-060142EB7BE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5559D041-469D-47B8-BF3C-E5A32646EB33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="461">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="462">
   <si>
     <t>Id</t>
   </si>
@@ -1411,6 +1411,9 @@
   </si>
   <si>
     <t>Traverse all edges, collect the number and find the sum. (node == null return, left shift OR combo, if it's a leaf add to the sum, else recur)</t>
+  </si>
+  <si>
+    <t>Sort Integers by The Number of 1 Bits</t>
   </si>
 </sst>
 </file>
@@ -1737,7 +1740,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G180"/>
+  <dimension ref="A1:G181"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -4270,6 +4273,17 @@
         <v>460</v>
       </c>
     </row>
+    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A181">
+        <v>1356</v>
+      </c>
+      <c r="B181" t="s">
+        <v>461</v>
+      </c>
+      <c r="C181" t="s">
+        <v>449</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G54">
     <sortCondition ref="A2:A54"/>

</xml_diff>

<commit_message>
Number Of Steps To Reduce A Number In Binary Representation To One.
</commit_message>
<xml_diff>
--- a/Pseudo.xlsx
+++ b/Pseudo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LC_Solutions\LC_Solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5559D041-469D-47B8-BF3C-E5A32646EB33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8949C6F-3F00-4E2A-8DFA-4A7922651EB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="462">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="465">
   <si>
     <t>Id</t>
   </si>
@@ -1414,6 +1414,15 @@
   </si>
   <si>
     <t>Sort Integers by The Number of 1 Bits</t>
+  </si>
+  <si>
+    <t>Number of Steps to Reduce a Number in Binary Representation to One</t>
+  </si>
+  <si>
+    <t>Count set bits and sort by lamda, or collect to group and sort each group and put back.</t>
+  </si>
+  <si>
+    <t>Use stringbuilder to simulate or just convert the char to int and do the last element check with carry. If it's an even step += 2, if it's odd step += 1</t>
   </si>
 </sst>
 </file>
@@ -1740,7 +1749,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G181"/>
+  <dimension ref="A1:G182"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -4283,6 +4292,23 @@
       <c r="C181" t="s">
         <v>449</v>
       </c>
+      <c r="D181" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A182">
+        <v>1404</v>
+      </c>
+      <c r="B182" t="s">
+        <v>462</v>
+      </c>
+      <c r="C182" t="s">
+        <v>449</v>
+      </c>
+      <c r="D182" t="s">
+        <v>464</v>
+      </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G54">

</xml_diff>

<commit_message>
Concatenation of Consecutive Binary Numbers.
</commit_message>
<xml_diff>
--- a/Pseudo.xlsx
+++ b/Pseudo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LC_Solutions\LC_Solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8949C6F-3F00-4E2A-8DFA-4A7922651EB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F2067F4-7642-476F-AD19-701039D7D803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="465">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="551" uniqueCount="467">
   <si>
     <t>Id</t>
   </si>
@@ -1422,7 +1422,13 @@
     <t>Count set bits and sort by lamda, or collect to group and sort each group and put back.</t>
   </si>
   <si>
-    <t>Use stringbuilder to simulate or just convert the char to int and do the last element check with carry. If it's an even step += 2, if it's odd step += 1</t>
+    <t>Use stringbuilder to simulate or just convert the char to int and do the last element check with carry. If (s[i] == '1' ? 1 : 0) + carry == 1 step += 2, else step += 1</t>
+  </si>
+  <si>
+    <t>Concatenation of Consecutive Binary Numbers</t>
+  </si>
+  <si>
+    <t>If I is power of 2 increase bit Length, Shift left by bitLengths and OR with i</t>
   </si>
 </sst>
 </file>
@@ -1749,7 +1755,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G182"/>
+  <dimension ref="A1:G183"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -4310,6 +4316,20 @@
         <v>464</v>
       </c>
     </row>
+    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A183">
+        <v>1680</v>
+      </c>
+      <c r="B183" t="s">
+        <v>465</v>
+      </c>
+      <c r="C183" t="s">
+        <v>449</v>
+      </c>
+      <c r="D183" t="s">
+        <v>466</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G54">
     <sortCondition ref="A2:A54"/>

</xml_diff>

<commit_message>
Partitioning Into Minimum Number of Deci-Binary Numbers.
</commit_message>
<xml_diff>
--- a/Pseudo.xlsx
+++ b/Pseudo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LC_Solutions\LC_Solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F2067F4-7642-476F-AD19-701039D7D803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A5A0A55-591B-4F7B-AE44-98057DFCA986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="551" uniqueCount="467">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="469">
   <si>
     <t>Id</t>
   </si>
@@ -1429,6 +1429,12 @@
   </si>
   <si>
     <t>If I is power of 2 increase bit Length, Shift left by bitLengths and OR with i</t>
+  </si>
+  <si>
+    <t>Partitioning Into Minimum Number of Deci-binary Numbers</t>
+  </si>
+  <si>
+    <t>each digit can be built by many 1s, find the max place value because we need that many terms of 1s to add up to it</t>
   </si>
 </sst>
 </file>
@@ -1755,7 +1761,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G183"/>
+  <dimension ref="A1:G184"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -4330,6 +4336,20 @@
         <v>466</v>
       </c>
     </row>
+    <row r="184" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A184">
+        <v>1689</v>
+      </c>
+      <c r="B184" t="s">
+        <v>467</v>
+      </c>
+      <c r="C184" t="s">
+        <v>97</v>
+      </c>
+      <c r="D184" t="s">
+        <v>468</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G54">
     <sortCondition ref="A2:A54"/>

</xml_diff>

<commit_message>
Minimum Swaps To Arrange A Binary Grid.
</commit_message>
<xml_diff>
--- a/Pseudo.xlsx
+++ b/Pseudo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LC_Solutions\LC_Solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A5A0A55-591B-4F7B-AE44-98057DFCA986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{237F5221-64B6-438E-BBB1-550645856594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="469">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="471">
   <si>
     <t>Id</t>
   </si>
@@ -1435,6 +1435,12 @@
   </si>
   <si>
     <t>each digit can be built by many 1s, find the max place value because we need that many terms of 1s to add up to it</t>
+  </si>
+  <si>
+    <t>Minimum Swaps to Arrange a Binary Grid</t>
+  </si>
+  <si>
+    <t>For each row find the rightmost index of 1 and store them in an [], simulate the swap by finding the row that has rightmost index 1 &lt;= current row I, if reaches n, impossible return -1, else swap they [] and bubbles it up</t>
   </si>
 </sst>
 </file>
@@ -1761,7 +1767,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G184"/>
+  <dimension ref="A1:G185"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -4350,6 +4356,20 @@
         <v>468</v>
       </c>
     </row>
+    <row r="185" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A185">
+        <v>1536</v>
+      </c>
+      <c r="B185" t="s">
+        <v>469</v>
+      </c>
+      <c r="C185" t="s">
+        <v>75</v>
+      </c>
+      <c r="D185" t="s">
+        <v>470</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G54">
     <sortCondition ref="A2:A54"/>

</xml_diff>

<commit_message>
Special Positions in A Binary Matrix.
</commit_message>
<xml_diff>
--- a/Pseudo.xlsx
+++ b/Pseudo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LC_Solutions\LC_Solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{237F5221-64B6-438E-BBB1-550645856594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA944D49-AD8D-4BC2-BDF8-71A4C5D65129}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="475">
   <si>
     <t>Id</t>
   </si>
@@ -1441,6 +1441,18 @@
   </si>
   <si>
     <t>For each row find the rightmost index of 1 and store them in an [], simulate the swap by finding the row that has rightmost index 1 &lt;= current row I, if reaches n, impossible return -1, else swap they [] and bubbles it up</t>
+  </si>
+  <si>
+    <t>Find Kth Bit in Nth Binary String</t>
+  </si>
+  <si>
+    <t>Math/Recursive</t>
+  </si>
+  <si>
+    <t>Special Positions in a Binary Matrix</t>
+  </si>
+  <si>
+    <t>Pass every cell to collect ones position, count ones on row and count ones on column. Pass thru the list of ones to see if the cell and row has ony 1 one.</t>
   </si>
 </sst>
 </file>
@@ -1767,7 +1779,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G185"/>
+  <dimension ref="A1:G187"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -4370,6 +4382,31 @@
         <v>470</v>
       </c>
     </row>
+    <row r="186" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A186">
+        <v>1545</v>
+      </c>
+      <c r="B186" t="s">
+        <v>471</v>
+      </c>
+      <c r="C186" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="187" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A187">
+        <v>1582</v>
+      </c>
+      <c r="B187" t="s">
+        <v>473</v>
+      </c>
+      <c r="C187" t="s">
+        <v>75</v>
+      </c>
+      <c r="D187" t="s">
+        <v>474</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G54">
     <sortCondition ref="A2:A54"/>

</xml_diff>

<commit_message>
Minimum Changes to Make Alternating Binary String.
</commit_message>
<xml_diff>
--- a/Pseudo.xlsx
+++ b/Pseudo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LC_Solutions\LC_Solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA944D49-AD8D-4BC2-BDF8-71A4C5D65129}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0E00069-59BA-4A90-8326-783E6BECE612}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="475">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="477">
   <si>
     <t>Id</t>
   </si>
@@ -1453,6 +1453,12 @@
   </si>
   <si>
     <t>Pass every cell to collect ones position, count ones on row and count ones on column. Pass thru the list of ones to see if the cell and row has ony 1 one.</t>
+  </si>
+  <si>
+    <t>Minimum Changes to Make Alternating Binary String</t>
+  </si>
+  <si>
+    <t>run 2 passes for 2 patterns or check even-odd index and return Math.Min(start0, s.Length - start0) very awesome.</t>
   </si>
 </sst>
 </file>
@@ -1779,7 +1785,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G187"/>
+  <dimension ref="A1:G188"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -4407,6 +4413,20 @@
         <v>474</v>
       </c>
     </row>
+    <row r="188" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A188">
+        <v>1758</v>
+      </c>
+      <c r="B188" t="s">
+        <v>475</v>
+      </c>
+      <c r="C188" t="s">
+        <v>75</v>
+      </c>
+      <c r="D188" t="s">
+        <v>476</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G54">
     <sortCondition ref="A2:A54"/>

</xml_diff>

<commit_message>
Check If Binray String Has At Most One Segment of Ones.
</commit_message>
<xml_diff>
--- a/Pseudo.xlsx
+++ b/Pseudo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LC_Solutions\LC_Solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0E00069-59BA-4A90-8326-783E6BECE612}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00ECCE94-B5F1-42EC-A292-8D96EE423741}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="477">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="479">
   <si>
     <t>Id</t>
   </si>
@@ -1459,6 +1459,12 @@
   </si>
   <si>
     <t>run 2 passes for 2 patterns or check even-odd index and return Math.Min(start0, s.Length - start0) very awesome.</t>
+  </si>
+  <si>
+    <t>Check if Binary String has at most one segment of ones</t>
+  </si>
+  <si>
+    <t>Check if there is a '0' then '1'.</t>
   </si>
 </sst>
 </file>
@@ -1785,7 +1791,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G188"/>
+  <dimension ref="A1:G189"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -4427,6 +4433,20 @@
         <v>476</v>
       </c>
     </row>
+    <row r="189" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A189">
+        <v>1784</v>
+      </c>
+      <c r="B189" t="s">
+        <v>477</v>
+      </c>
+      <c r="C189" t="s">
+        <v>75</v>
+      </c>
+      <c r="D189" t="s">
+        <v>478</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G54">
     <sortCondition ref="A2:A54"/>

</xml_diff>

<commit_message>
Minimum Number of Flips to Make the Binary String Alternating.
</commit_message>
<xml_diff>
--- a/Pseudo.xlsx
+++ b/Pseudo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LC_Solutions\LC_Solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00ECCE94-B5F1-42EC-A292-8D96EE423741}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{663AE30F-C7F0-4E25-9DA0-E5103BC65225}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="479">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="480">
   <si>
     <t>Id</t>
   </si>
@@ -1465,6 +1465,9 @@
   </si>
   <si>
     <t>Check if there is a '0' then '1'.</t>
+  </si>
+  <si>
+    <t>Minimum Number of Flips to Make the Binary String alternating</t>
   </si>
 </sst>
 </file>
@@ -1791,7 +1794,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G189"/>
+  <dimension ref="A1:G190"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -4447,6 +4450,17 @@
         <v>478</v>
       </c>
     </row>
+    <row r="190" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A190">
+        <v>1888</v>
+      </c>
+      <c r="B190" t="s">
+        <v>479</v>
+      </c>
+      <c r="C190" t="s">
+        <v>75</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G54">
     <sortCondition ref="A2:A54"/>

</xml_diff>

<commit_message>
Find Unique Binary String.
</commit_message>
<xml_diff>
--- a/Pseudo.xlsx
+++ b/Pseudo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LC_Solutions\LC_Solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{663AE30F-C7F0-4E25-9DA0-E5103BC65225}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{762C59A9-7804-4774-AC3E-9579846E1685}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="480">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="483">
   <si>
     <t>Id</t>
   </si>
@@ -1468,6 +1468,15 @@
   </si>
   <si>
     <t>Minimum Number of Flips to Make the Binary String alternating</t>
+  </si>
+  <si>
+    <t>Find Unique Binary String</t>
+  </si>
+  <si>
+    <t>Math/Loop/Recursive</t>
+  </si>
+  <si>
+    <t>Cantor's Diagnol Trick OR convert all into int, find the missing int and convert back</t>
   </si>
 </sst>
 </file>
@@ -1794,7 +1803,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G190"/>
+  <dimension ref="A1:G191"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -4461,6 +4470,20 @@
         <v>75</v>
       </c>
     </row>
+    <row r="191" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A191">
+        <v>1980</v>
+      </c>
+      <c r="B191" t="s">
+        <v>480</v>
+      </c>
+      <c r="C191" t="s">
+        <v>481</v>
+      </c>
+      <c r="D191" t="s">
+        <v>482</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G54">
     <sortCondition ref="A2:A54"/>

</xml_diff>

<commit_message>
Complement Of Base 10 Integer.
</commit_message>
<xml_diff>
--- a/Pseudo.xlsx
+++ b/Pseudo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LC_Solutions\LC_Solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{762C59A9-7804-4774-AC3E-9579846E1685}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5012A8EF-69F6-4AB6-9D48-843F9F3B0BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="483">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="487">
   <si>
     <t>Id</t>
   </si>
@@ -1477,6 +1477,18 @@
   </si>
   <si>
     <t>Cantor's Diagnol Trick OR convert all into int, find the missing int and convert back</t>
+  </si>
+  <si>
+    <t>Find All Possible Stable Binary Arrays 1</t>
+  </si>
+  <si>
+    <t>Complement of Base 10 Integer</t>
+  </si>
+  <si>
+    <t>Math/Bitwise/Loop</t>
+  </si>
+  <si>
+    <t>extract last bit, flip, left shift the flip based on the current iteration for msb, OR the complement with the flip until n = 0</t>
   </si>
 </sst>
 </file>
@@ -1803,7 +1815,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G191"/>
+  <dimension ref="A1:G193"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -4484,6 +4496,31 @@
         <v>482</v>
       </c>
     </row>
+    <row r="192" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A192">
+        <v>3129</v>
+      </c>
+      <c r="B192" t="s">
+        <v>483</v>
+      </c>
+      <c r="C192" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="193" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A193">
+        <v>1009</v>
+      </c>
+      <c r="B193" t="s">
+        <v>484</v>
+      </c>
+      <c r="C193" t="s">
+        <v>485</v>
+      </c>
+      <c r="D193" t="s">
+        <v>486</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G54">
     <sortCondition ref="A2:A54"/>

</xml_diff>

<commit_message>
Minimum Number Of Seconds To Make Mountain Height Zero.
</commit_message>
<xml_diff>
--- a/Pseudo.xlsx
+++ b/Pseudo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LC_Solutions\LC_Solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5012A8EF-69F6-4AB6-9D48-843F9F3B0BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{565DAD24-2485-4DE8-AC56-B20EE48CDFC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="487">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="581" uniqueCount="490">
   <si>
     <t>Id</t>
   </si>
@@ -1489,6 +1489,15 @@
   </si>
   <si>
     <t>extract last bit, flip, left shift the flip based on the current iteration for msb, OR the complement with the flip until n = 0</t>
+  </si>
+  <si>
+    <t>Minimum Number of Seconds to Make Mountain Height Zero</t>
+  </si>
+  <si>
+    <t>Math/Loop/Binary Search</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use inequality to find the formulat for the height can be removed by each worker at each time, make a helper function to check if it can be finished. Use Binary search to find time from left = 0 to right = max time (arithmetic sum time * height(height+1)/2) a weakest worker can do. </t>
   </si>
 </sst>
 </file>
@@ -1815,7 +1824,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G193"/>
+  <dimension ref="A1:G194"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -4521,6 +4530,20 @@
         <v>486</v>
       </c>
     </row>
+    <row r="194" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A194">
+        <v>3296</v>
+      </c>
+      <c r="B194" t="s">
+        <v>487</v>
+      </c>
+      <c r="C194" t="s">
+        <v>488</v>
+      </c>
+      <c r="D194" t="s">
+        <v>489</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G54">
     <sortCondition ref="A2:A54"/>

</xml_diff>

<commit_message>
The K_th Lexicographical String Of All Happy Strings Of Length N.
</commit_message>
<xml_diff>
--- a/Pseudo.xlsx
+++ b/Pseudo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LC_Solutions\LC_Solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{565DAD24-2485-4DE8-AC56-B20EE48CDFC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10F5DC9D-7C68-4A09-993C-7EB4F33A0E9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="581" uniqueCount="490">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="584" uniqueCount="492">
   <si>
     <t>Id</t>
   </si>
@@ -1498,6 +1498,12 @@
   </si>
   <si>
     <t xml:space="preserve">Use inequality to find the formulat for the height can be removed by each worker at each time, make a helper function to check if it can be finished. Use Binary search to find time from left = 0 to right = max time (arithmetic sum time * height(height+1)/2) a weakest worker can do. </t>
+  </si>
+  <si>
+    <t>The K_th Lexicographical String Of All Happy Strings Of Length N</t>
+  </si>
+  <si>
+    <t>Recursively build the strings and then return the item k-1 in the List OR keep building and tracking the current count until it reaches n.</t>
   </si>
 </sst>
 </file>
@@ -1824,7 +1830,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G194"/>
+  <dimension ref="A1:G195"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -4544,6 +4550,20 @@
         <v>489</v>
       </c>
     </row>
+    <row r="195" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A195">
+        <v>1415</v>
+      </c>
+      <c r="B195" t="s">
+        <v>490</v>
+      </c>
+      <c r="C195" t="s">
+        <v>481</v>
+      </c>
+      <c r="D195" t="s">
+        <v>491</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G54">
     <sortCondition ref="A2:A54"/>

</xml_diff>

<commit_message>
Largest Submatrix With Rearrangements.
</commit_message>
<xml_diff>
--- a/Pseudo.xlsx
+++ b/Pseudo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LC_Solutions\LC_Solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22B72F34-3722-41E8-98EC-0C45817F2662}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F609958F-BB33-401D-93A6-0321A9F05E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="494">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="498">
   <si>
     <t>Id</t>
   </si>
@@ -1510,6 +1510,18 @@
   </si>
   <si>
     <t>Class Implementation</t>
+  </si>
+  <si>
+    <t>Get Biggest Three Rhombus Sums in a Grid</t>
+  </si>
+  <si>
+    <t>Math/Loop/HashSet</t>
+  </si>
+  <si>
+    <t>Go thru each cell, find sums of all possible rhombus, return top 3 highest OrderByDescending</t>
+  </si>
+  <si>
+    <t>Largest Submatrix With Rearrangements</t>
   </si>
 </sst>
 </file>
@@ -1836,7 +1848,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G196"/>
+  <dimension ref="A1:G198"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -4581,6 +4593,28 @@
         <v>493</v>
       </c>
     </row>
+    <row r="197" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A197">
+        <v>1878</v>
+      </c>
+      <c r="B197" t="s">
+        <v>494</v>
+      </c>
+      <c r="C197" t="s">
+        <v>495</v>
+      </c>
+      <c r="D197" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="198" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A198">
+        <v>1727</v>
+      </c>
+      <c r="B198" t="s">
+        <v>497</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G54">
     <sortCondition ref="A2:A54"/>

</xml_diff>

<commit_message>
Count Submatrices with Top Left Element and Sum Less Than K.
</commit_message>
<xml_diff>
--- a/Pseudo.xlsx
+++ b/Pseudo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LC_Solutions\LC_Solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F609958F-BB33-401D-93A6-0321A9F05E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{616C5C31-0156-4A88-BFF7-5750DF917EFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="498">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="501">
   <si>
     <t>Id</t>
   </si>
@@ -1522,6 +1522,15 @@
   </si>
   <si>
     <t>Largest Submatrix With Rearrangements</t>
+  </si>
+  <si>
+    <t>Have a prefixSum for each row(modify the row with the consecutive ones from prev row), then order by descending and do histogram area, first col is 1, second col is 2, etc. for finding the max for each cell</t>
+  </si>
+  <si>
+    <t>Count Submatrices with Top-Left Element and Sum Less Than k</t>
+  </si>
+  <si>
+    <t>PrefixSum left to right, top to bottom for each cell, because all the cell are positive, obviously top left is less than k when sum is less than or equal to K.</t>
   </si>
 </sst>
 </file>
@@ -1848,7 +1857,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G198"/>
+  <dimension ref="A1:G199"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -4614,6 +4623,26 @@
       <c r="B198" t="s">
         <v>497</v>
       </c>
+      <c r="C198" t="s">
+        <v>75</v>
+      </c>
+      <c r="D198" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="199" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A199">
+        <v>3070</v>
+      </c>
+      <c r="B199" t="s">
+        <v>499</v>
+      </c>
+      <c r="C199" t="s">
+        <v>75</v>
+      </c>
+      <c r="D199" t="s">
+        <v>500</v>
+      </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G54">

</xml_diff>

<commit_message>
Count Submatrices with Equal Frequency Of X and Y.
</commit_message>
<xml_diff>
--- a/Pseudo.xlsx
+++ b/Pseudo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LC_Solutions\LC_Solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{616C5C31-0156-4A88-BFF7-5750DF917EFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9559135-6F13-4C1B-A810-6FF0303660E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="501">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="598" uniqueCount="503">
   <si>
     <t>Id</t>
   </si>
@@ -1531,6 +1531,12 @@
   </si>
   <si>
     <t>PrefixSum left to right, top to bottom for each cell, because all the cell are positive, obviously top left is less than k when sum is less than or equal to K.</t>
+  </si>
+  <si>
+    <t>Count Submatrices with Equal Frequency of X and Y</t>
+  </si>
+  <si>
+    <t>PrefixX and prefixY, iterate thru each cell and count x and y. if they're equal and there is at least 1 x then add to the count.</t>
   </si>
 </sst>
 </file>
@@ -1857,7 +1863,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G199"/>
+  <dimension ref="A1:G200"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -4644,6 +4650,20 @@
         <v>500</v>
       </c>
     </row>
+    <row r="200" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A200">
+        <v>3212</v>
+      </c>
+      <c r="B200" t="s">
+        <v>501</v>
+      </c>
+      <c r="C200" t="s">
+        <v>75</v>
+      </c>
+      <c r="D200" t="s">
+        <v>502</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G54">
     <sortCondition ref="A2:A54"/>

</xml_diff>

<commit_message>
Find Square Submatrix Vertically.
</commit_message>
<xml_diff>
--- a/Pseudo.xlsx
+++ b/Pseudo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LC_Solutions\LC_Solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9559135-6F13-4C1B-A810-6FF0303660E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{025F880F-66C3-469D-A94F-A9EA6F9B93E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="598" uniqueCount="503">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="504">
   <si>
     <t>Id</t>
   </si>
@@ -1537,6 +1537,9 @@
   </si>
   <si>
     <t>PrefixX and prefixY, iterate thru each cell and count x and y. if they're equal and there is at least 1 x then add to the count.</t>
+  </si>
+  <si>
+    <t>Flip Square Submatrix Vertically</t>
   </si>
 </sst>
 </file>
@@ -1863,7 +1866,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G200"/>
+  <dimension ref="A1:G201"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -4664,6 +4667,17 @@
         <v>502</v>
       </c>
     </row>
+    <row r="201" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A201">
+        <v>3643</v>
+      </c>
+      <c r="B201" t="s">
+        <v>503</v>
+      </c>
+      <c r="C201" t="s">
+        <v>97</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G54">
     <sortCondition ref="A2:A54"/>

</xml_diff>

<commit_message>
Determine Whether a Matrix Can Be Obtained By Rotation.
</commit_message>
<xml_diff>
--- a/Pseudo.xlsx
+++ b/Pseudo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LC_Solutions\LC_Solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{025F880F-66C3-469D-A94F-A9EA6F9B93E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{755BDBD4-276B-4E0F-91CD-0CAF9D0D696D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="504">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="507">
   <si>
     <t>Id</t>
   </si>
@@ -1540,6 +1540,15 @@
   </si>
   <si>
     <t>Flip Square Submatrix Vertically</t>
+  </si>
+  <si>
+    <t>Iterate and swap [x + k - i - 1][y+j]</t>
+  </si>
+  <si>
+    <t>Determine Whether a Matrix Can Be Obtained By Roation</t>
+  </si>
+  <si>
+    <t>rotated[i][j] = mat[n - j - 1][i];</t>
   </si>
 </sst>
 </file>
@@ -1866,7 +1875,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G201"/>
+  <dimension ref="A1:G202"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -4675,7 +4684,24 @@
         <v>503</v>
       </c>
       <c r="C201" t="s">
-        <v>97</v>
+        <v>75</v>
+      </c>
+      <c r="D201" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="202" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A202">
+        <v>1886</v>
+      </c>
+      <c r="B202" t="s">
+        <v>505</v>
+      </c>
+      <c r="C202" t="s">
+        <v>75</v>
+      </c>
+      <c r="D202" t="s">
+        <v>506</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Maximum Non Negative Product In a Matrix.
</commit_message>
<xml_diff>
--- a/Pseudo.xlsx
+++ b/Pseudo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LC_Solutions\LC_Solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{755BDBD4-276B-4E0F-91CD-0CAF9D0D696D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22678F9A-A2B5-4100-B792-0E291D1D2256}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="507">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="510">
   <si>
     <t>Id</t>
   </si>
@@ -1549,6 +1549,15 @@
   </si>
   <si>
     <t>rotated[i][j] = mat[n - j - 1][i];</t>
+  </si>
+  <si>
+    <t>Maximum Non Negative Product in a Matrix</t>
+  </si>
+  <si>
+    <t>Math/Loop/Dynamic Programming</t>
+  </si>
+  <si>
+    <t>minDp, maxDp, right and down, 4 candidates, result is the maxDp[m-1,n-1]</t>
   </si>
 </sst>
 </file>
@@ -1875,7 +1884,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G202"/>
+  <dimension ref="A1:G203"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -4704,6 +4713,20 @@
         <v>506</v>
       </c>
     </row>
+    <row r="203" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A203">
+        <v>1594</v>
+      </c>
+      <c r="B203" t="s">
+        <v>507</v>
+      </c>
+      <c r="C203" t="s">
+        <v>508</v>
+      </c>
+      <c r="D203" t="s">
+        <v>509</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G54">
     <sortCondition ref="A2:A54"/>

</xml_diff>

<commit_message>
Equal Sum Grid Partition 1.
</commit_message>
<xml_diff>
--- a/Pseudo.xlsx
+++ b/Pseudo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LC_Solutions\LC_Solutions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72F303E5-9884-44E5-A1F8-C8646BEC0539}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4186F38B-7FF6-4989-883D-3C1BA425E843}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="610" uniqueCount="513">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="613" uniqueCount="516">
   <si>
     <t>Id</t>
   </si>
@@ -1567,6 +1567,15 @@
   </si>
   <si>
     <t>Have prefixProduct and suffixProduct, flatten the matrix, iterate from the last element and change the suffix accordingly, current value = prefix * suffix then apply modular.</t>
+  </si>
+  <si>
+    <t>Equal Sum Grid Partition 1</t>
+  </si>
+  <si>
+    <t>Math/Loop/Prefix</t>
+  </si>
+  <si>
+    <t>Find the total, see if it's even, have a prefix, passing the matrix twice to see if there is an even half?</t>
   </si>
 </sst>
 </file>
@@ -1893,7 +1902,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G204"/>
+  <dimension ref="A1:G205"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
@@ -4750,6 +4759,20 @@
         <v>512</v>
       </c>
     </row>
+    <row r="205" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A205">
+        <v>3546</v>
+      </c>
+      <c r="B205" t="s">
+        <v>513</v>
+      </c>
+      <c r="C205" t="s">
+        <v>514</v>
+      </c>
+      <c r="D205" t="s">
+        <v>515</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G54">
     <sortCondition ref="A2:A54"/>

</xml_diff>